<commit_message>
revised for 2026 submission. Added reproduced results from SGSLAM NGDSLAM PanopticSLAM.
</commit_message>
<xml_diff>
--- a/Examples/RGB-D/results/2025-revised-result/ROVK-SLAM-result.xlsx
+++ b/Examples/RGB-D/results/2025-revised-result/ROVK-SLAM-result.xlsx
@@ -21453,34 +21453,34 @@
       <c r="M258" s="9" t="n">
         <v>0.019157</v>
       </c>
-      <c r="N258" s="0" t="n">
+      <c r="N258" s="9" t="n">
         <v>0.017272</v>
       </c>
-      <c r="O258" s="0" t="n">
+      <c r="O258" s="9" t="n">
         <v>0.018461</v>
       </c>
-      <c r="P258" s="0" t="n">
+      <c r="P258" s="9" t="n">
         <v>0.018788</v>
       </c>
-      <c r="Q258" s="0" t="n">
+      <c r="Q258" s="9" t="n">
         <v>0.017028</v>
       </c>
-      <c r="R258" s="0" t="n">
+      <c r="R258" s="9" t="n">
         <v>0.017268</v>
       </c>
-      <c r="S258" s="0" t="n">
+      <c r="S258" s="9" t="n">
         <v>0.017016</v>
       </c>
-      <c r="T258" s="0" t="n">
+      <c r="T258" s="9" t="n">
         <v>0.017856</v>
       </c>
-      <c r="U258" s="0" t="n">
+      <c r="U258" s="9" t="n">
         <v>0.017617</v>
       </c>
-      <c r="V258" s="0" t="n">
+      <c r="V258" s="9" t="n">
         <v>0.017172</v>
       </c>
-      <c r="W258" s="0" t="n">
+      <c r="W258" s="9" t="n">
         <v>0.017322</v>
       </c>
     </row>

</xml_diff>